<commit_message>
Study materials, exam sections, students list
</commit_message>
<xml_diff>
--- a/sample-questions.xlsx
+++ b/sample-questions.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:G7"/>
   <cols>
     <col min="1" max="1" width="70.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -405,6 +405,7 @@
     <col min="4" max="4" width="14.83203125" customWidth="1"/>
     <col min="5" max="5" width="14.83203125" customWidth="1"/>
     <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -426,6 +427,9 @@
       <c r="F1" t="str">
         <v>Correct</v>
       </c>
+      <c r="G1" t="str">
+        <v>Section</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -446,6 +450,9 @@
       <c r="F2" t="str">
         <v>C</v>
       </c>
+      <c r="G2" t="str">
+        <v>Aptitude</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -466,6 +473,9 @@
       <c r="F3" t="str">
         <v>C</v>
       </c>
+      <c r="G3" t="str">
+        <v>Aptitude</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -486,6 +496,9 @@
       <c r="F4" t="str">
         <v>B</v>
       </c>
+      <c r="G4" t="str">
+        <v>Aptitude</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -506,30 +519,59 @@
       <c r="F5" t="str">
         <v>B</v>
       </c>
+      <c r="G5" t="str">
+        <v>Reasoning</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
+        <v>If CAT is coded as 3120, how is DOG coded?</v>
+      </c>
+      <c r="B6" t="str">
+        <v>4157</v>
+      </c>
+      <c r="C6" t="str">
+        <v>41507</v>
+      </c>
+      <c r="D6" t="str">
+        <v>4057</v>
+      </c>
+      <c r="E6" t="str">
+        <v>415</v>
+      </c>
+      <c r="F6" t="str">
+        <v>B</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Reasoning</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
         <v>The average of 5 numbers is 20. If one number is excluded, the average becomes 18. The excluded number is:</v>
       </c>
-      <c r="B6" t="str">
+      <c r="B7" t="str">
         <v>24</v>
       </c>
-      <c r="C6" t="str">
+      <c r="C7" t="str">
         <v>26</v>
       </c>
-      <c r="D6" t="str">
+      <c r="D7" t="str">
         <v>28</v>
       </c>
-      <c r="E6" t="str">
+      <c r="E7" t="str">
         <v>30</v>
       </c>
-      <c r="F6" t="str">
+      <c r="F7" t="str">
         <v>C</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Aptitude</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>